<commit_message>
Notebook 10 : prévision des ventes, src/modeles.py
</commit_message>
<xml_diff>
--- a/reports/livrables/L1_L2_phases_backlog/dictionnaire_donnees.xlsx
+++ b/reports/livrables/L1_L2_phases_backlog/dictionnaire_donnees.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ventes" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dimensions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contrôle dimensions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liens dimensions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Utilisation dimensions" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fichiers" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Correspondance clés" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Autres tables de faits" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lignes par année" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recoupement des ventes" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FactStrategyPlan" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FactSalesQuota" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FactInventory" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FactOnlineSales" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Ventes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dimensions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Contrôle dimensions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Liens dimensions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Utilisation dimensions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Fichiers" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Correspondance clés" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Autres tables de faits" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Lignes par année" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Recoupement des ventes" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="FactStrategyPlan" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="FactSalesQuota" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="FactInventory" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="FactOnlineSales" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>